<commit_message>
feat: 439 - modals and misc. (#489)
* initial commit

* second commit

* third commit

* fourth commit

* fifth commit
</commit_message>
<xml_diff>
--- a/next/app/compliance-reporting/lib/model-year-reports/templates/model_year_report_template.xlsx
+++ b/next/app/compliance-reporting/lib/model-year-reports/templates/model_year_report_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timchen/Desktop/zeva/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6A8444E-2219-8741-B40C-B46472DD4034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE204FB8-C6E6-4E4A-AFD1-50B984D79033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3600" yWindow="1660" windowWidth="28040" windowHeight="17440" xr2:uid="{19A56954-7A74-5647-9FDF-D514421742EB}"/>
   </bookViews>
@@ -17,13 +17,14 @@
     <sheet name="Previous Volumes" sheetId="14" r:id="rId2"/>
     <sheet name="Vehicle Statistics" sheetId="3" r:id="rId3"/>
     <sheet name="Compliance Ratio Reductions" sheetId="7" r:id="rId4"/>
-    <sheet name="Beginning Balance" sheetId="4" r:id="rId5"/>
-    <sheet name="Credits" sheetId="9" r:id="rId6"/>
-    <sheet name="Pending Supply Credits" sheetId="15" r:id="rId7"/>
-    <sheet name="Adjustments" sheetId="16" r:id="rId8"/>
-    <sheet name="Suggested Adjustments" sheetId="17" r:id="rId9"/>
-    <sheet name="Offsets and Transfers Away" sheetId="8" r:id="rId10"/>
-    <sheet name="Preliminary Ending Balance" sheetId="13" r:id="rId11"/>
+    <sheet name="Balance at end of prev CD" sheetId="18" r:id="rId5"/>
+    <sheet name="Balance after prev CD" sheetId="4" r:id="rId6"/>
+    <sheet name="Credits" sheetId="9" r:id="rId7"/>
+    <sheet name="Pending Supply Credits" sheetId="15" r:id="rId8"/>
+    <sheet name="Adjustments" sheetId="16" r:id="rId9"/>
+    <sheet name="Suggested Adjustments" sheetId="17" r:id="rId10"/>
+    <sheet name="Offsets and Transfers Away" sheetId="8" r:id="rId11"/>
+    <sheet name="Preliminary Ending Balance" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="22">
   <si>
     <t>Vehicle Class</t>
   </si>
@@ -527,6 +528,39 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93202DF-651A-F84D-B1EE-4F20F874319C}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.1640625" customWidth="1"/>
+    <col min="3" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC33D11-4CAF-4F4A-92DA-707B8A2A3658}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -560,7 +594,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93F66F5F-C88E-1542-A176-3B58C5328BD4}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -707,6 +741,40 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A01E355-090E-B543-A3E2-86E0C2E836F4}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" customWidth="1"/>
+    <col min="5" max="5" width="21.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68F82AF4-275E-A740-B0B8-C2E446D618C6}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -739,7 +807,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4F086B9-ACA4-F148-854C-0618C5A00B58}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -773,7 +841,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{899E1038-FF57-F54A-A9F3-6C033DF5A336}">
   <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -803,7 +871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6DEF3C0-3EAE-A44C-B7E1-AE086C8F392C}">
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -835,37 +903,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93202DF-651A-F84D-B1EE-4F20F874319C}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="18.83203125" customWidth="1"/>
-    <col min="2" max="2" width="21.1640625" customWidth="1"/>
-    <col min="3" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>